<commit_message>
data: regenera apuracao_q4_exportado com novos clientes
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/apuracao_q4_exportado.xlsx
+++ b/backend/apuracao_q4_exportado.xlsx
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>67180.22</v>
+        <v>127180.22</v>
       </c>
     </row>
     <row r="38">
@@ -1385,7 +1385,7 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>-42323.54</v>
+        <v>-80123.53999999999</v>
       </c>
     </row>
     <row r="39">
@@ -1410,7 +1410,7 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>24856.68</v>
+        <v>47056.68</v>
       </c>
     </row>
     <row r="40">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>6224535.49</v>
+        <v>6284535.49</v>
       </c>
     </row>
     <row r="41">
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>-2894465.03</v>
+        <v>-2932265.03</v>
       </c>
     </row>
     <row r="42">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>3330070.46</v>
+        <v>3352270.46</v>
       </c>
     </row>
     <row r="43">
@@ -7635,7 +7635,7 @@
         </is>
       </c>
       <c r="E288" s="2" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="289">
@@ -7660,7 +7660,7 @@
         </is>
       </c>
       <c r="E289" s="2" t="n">
-        <v>-0</v>
+        <v>-18900</v>
       </c>
     </row>
     <row r="290">
@@ -7685,7 +7685,7 @@
         </is>
       </c>
       <c r="E290" s="2" t="n">
-        <v>0</v>
+        <v>11100</v>
       </c>
     </row>
     <row r="291">
@@ -7710,7 +7710,7 @@
         </is>
       </c>
       <c r="E291" s="2" t="n">
-        <v>2456502.71</v>
+        <v>2486502.71</v>
       </c>
     </row>
     <row r="292">
@@ -7735,7 +7735,7 @@
         </is>
       </c>
       <c r="E292" s="2" t="n">
-        <v>-713853.33</v>
+        <v>-732753.33</v>
       </c>
     </row>
     <row r="293">
@@ -7760,7 +7760,7 @@
         </is>
       </c>
       <c r="E293" s="2" t="n">
-        <v>1742649.38</v>
+        <v>1753749.38</v>
       </c>
     </row>
     <row r="294">
@@ -7785,7 +7785,7 @@
         </is>
       </c>
       <c r="E294" s="2" t="n">
-        <v>1742649.38</v>
+        <v>1753749.38</v>
       </c>
     </row>
     <row r="295">
@@ -7885,7 +7885,7 @@
         </is>
       </c>
       <c r="E298" s="2" t="n">
-        <v>4015041.7</v>
+        <v>4114791.7</v>
       </c>
     </row>
     <row r="299">
@@ -7935,7 +7935,7 @@
         </is>
       </c>
       <c r="E300" s="2" t="n">
-        <v>1424309.39</v>
+        <v>1524059.39</v>
       </c>
     </row>
     <row r="301">
@@ -8185,7 +8185,7 @@
         </is>
       </c>
       <c r="E310" s="2" t="n">
-        <v>4015041.7</v>
+        <v>4114791.7</v>
       </c>
     </row>
     <row r="311">
@@ -8235,7 +8235,7 @@
         </is>
       </c>
       <c r="E312" s="2" t="n">
-        <v>1424309.39</v>
+        <v>1524059.39</v>
       </c>
     </row>
     <row r="313">
@@ -8260,7 +8260,7 @@
         </is>
       </c>
       <c r="E313" s="2" t="n">
-        <v>1424309.39</v>
+        <v>1524059.39</v>
       </c>
     </row>
     <row r="314">
@@ -9635,7 +9635,7 @@
         </is>
       </c>
       <c r="E368" s="2" t="n">
-        <v>0</v>
+        <v>292500</v>
       </c>
     </row>
     <row r="369">
@@ -9660,7 +9660,7 @@
         </is>
       </c>
       <c r="E369" s="2" t="n">
-        <v>-0</v>
+        <v>-184275</v>
       </c>
     </row>
     <row r="370">
@@ -9685,7 +9685,7 @@
         </is>
       </c>
       <c r="E370" s="2" t="n">
-        <v>0</v>
+        <v>108225</v>
       </c>
     </row>
     <row r="371">
@@ -9710,7 +9710,7 @@
         </is>
       </c>
       <c r="E371" s="2" t="n">
-        <v>3685754.45</v>
+        <v>3978254.45</v>
       </c>
     </row>
     <row r="372">
@@ -9735,7 +9735,7 @@
         </is>
       </c>
       <c r="E372" s="2" t="n">
-        <v>-2144384.8</v>
+        <v>-2328659.8</v>
       </c>
     </row>
     <row r="373">
@@ -9760,7 +9760,7 @@
         </is>
       </c>
       <c r="E373" s="2" t="n">
-        <v>1541369.65</v>
+        <v>1649594.65</v>
       </c>
     </row>
     <row r="374">
@@ -9785,7 +9785,7 @@
         </is>
       </c>
       <c r="E374" s="2" t="n">
-        <v>1541369.65</v>
+        <v>1649594.65</v>
       </c>
     </row>
     <row r="375">
@@ -10110,7 +10110,7 @@
         </is>
       </c>
       <c r="E387" s="2" t="n">
-        <v>1904136.13</v>
+        <v>2048400.13</v>
       </c>
     </row>
     <row r="388">
@@ -10135,7 +10135,7 @@
         </is>
       </c>
       <c r="E388" s="2" t="n">
-        <v>-1199605.76</v>
+        <v>-1290492.08</v>
       </c>
     </row>
     <row r="389">
@@ -10160,7 +10160,7 @@
         </is>
       </c>
       <c r="E389" s="2" t="n">
-        <v>704530.37</v>
+        <v>757908.05</v>
       </c>
     </row>
     <row r="390">
@@ -10185,7 +10185,7 @@
         </is>
       </c>
       <c r="E390" s="2" t="n">
-        <v>11536823.97</v>
+        <v>11681087.97</v>
       </c>
     </row>
     <row r="391">
@@ -10210,7 +10210,7 @@
         </is>
       </c>
       <c r="E391" s="2" t="n">
-        <v>-6931058.52</v>
+        <v>-7021944.84</v>
       </c>
     </row>
     <row r="392">
@@ -10235,7 +10235,7 @@
         </is>
       </c>
       <c r="E392" s="2" t="n">
-        <v>4605765.45</v>
+        <v>4659143.13</v>
       </c>
     </row>
     <row r="393">
@@ -10685,7 +10685,7 @@
         </is>
       </c>
       <c r="E410" s="2" t="n">
-        <v>215580.48</v>
+        <v>359844.48</v>
       </c>
     </row>
     <row r="411">
@@ -10710,7 +10710,7 @@
         </is>
       </c>
       <c r="E411" s="2" t="n">
-        <v>-32451.8</v>
+        <v>-123338.12</v>
       </c>
     </row>
     <row r="412">
@@ -10735,7 +10735,7 @@
         </is>
       </c>
       <c r="E412" s="2" t="n">
-        <v>183128.68</v>
+        <v>236506.36</v>
       </c>
     </row>
     <row r="413">
@@ -10760,7 +10760,7 @@
         </is>
       </c>
       <c r="E413" s="2" t="n">
-        <v>4760893.7</v>
+        <v>4905157.7</v>
       </c>
     </row>
     <row r="414">
@@ -10785,7 +10785,7 @@
         </is>
       </c>
       <c r="E414" s="2" t="n">
-        <v>-3086440.63</v>
+        <v>-3177326.95</v>
       </c>
     </row>
     <row r="415">
@@ -10810,7 +10810,7 @@
         </is>
       </c>
       <c r="E415" s="2" t="n">
-        <v>1674453.07</v>
+        <v>1727830.75</v>
       </c>
     </row>
     <row r="416">
@@ -10835,7 +10835,7 @@
         </is>
       </c>
       <c r="E416" s="2" t="n">
-        <v>1674453.07</v>
+        <v>1727830.75</v>
       </c>
     </row>
     <row r="417">
@@ -12110,7 +12110,7 @@
         </is>
       </c>
       <c r="E467" s="2" t="n">
-        <v>0</v>
+        <v>684750</v>
       </c>
     </row>
     <row r="468">
@@ -12135,7 +12135,7 @@
         </is>
       </c>
       <c r="E468" s="2" t="n">
-        <v>-0</v>
+        <v>-431392.5</v>
       </c>
     </row>
     <row r="469">
@@ -12160,7 +12160,7 @@
         </is>
       </c>
       <c r="E469" s="2" t="n">
-        <v>0</v>
+        <v>253357.5</v>
       </c>
     </row>
     <row r="470">
@@ -12185,7 +12185,7 @@
         </is>
       </c>
       <c r="E470" s="2" t="n">
-        <v>13825143.05</v>
+        <v>14509893.05</v>
       </c>
     </row>
     <row r="471">
@@ -12210,7 +12210,7 @@
         </is>
       </c>
       <c r="E471" s="2" t="n">
-        <v>-8779281.42</v>
+        <v>-9210673.92</v>
       </c>
     </row>
     <row r="472">
@@ -12235,7 +12235,7 @@
         </is>
       </c>
       <c r="E472" s="2" t="n">
-        <v>5045861.63</v>
+        <v>5299219.13</v>
       </c>
     </row>
     <row r="473">

</xml_diff>

<commit_message>
fix: LB usa marg_by_client (mesmo da aba margem por cliente)
Antes o LB usava lb_visual = RAC - |custo|, misturando fontes distintas
e inflando clientes com custo=0 mas RAC > receita_margem (ex: BUNZL
mostrava 186k em vez de 130k que aparece na aba margem por cliente).

Agora both clientes_detalhe e detalhe_ws usam marg_by_client /
actual_marg_ws diretamente do margem_projetos.csv, a mesma fonte da aba
margem por cliente.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/apuracao_q4_exportado.xlsx
+++ b/backend/apuracao_q4_exportado.xlsx
@@ -4110,7 +4110,7 @@
         </is>
       </c>
       <c r="E147" s="2" t="n">
-        <v>-1426517.06</v>
+        <v>-1469800.85</v>
       </c>
     </row>
     <row r="148">
@@ -4135,7 +4135,7 @@
         </is>
       </c>
       <c r="E148" s="2" t="n">
-        <v>1215122.15</v>
+        <v>1171838.36</v>
       </c>
     </row>
     <row r="149">
@@ -4410,7 +4410,7 @@
         </is>
       </c>
       <c r="E159" s="2" t="n">
-        <v>-1426517.06</v>
+        <v>-1469800.85</v>
       </c>
     </row>
     <row r="160">
@@ -4435,7 +4435,7 @@
         </is>
       </c>
       <c r="E160" s="2" t="n">
-        <v>1215122.15</v>
+        <v>1171838.36</v>
       </c>
     </row>
     <row r="161">
@@ -4460,7 +4460,7 @@
         </is>
       </c>
       <c r="E161" s="2" t="n">
-        <v>1215122.15</v>
+        <v>1171838.36</v>
       </c>
     </row>
     <row r="162">
@@ -4585,7 +4585,7 @@
         </is>
       </c>
       <c r="E166" s="2" t="n">
-        <v>-1430318.25</v>
+        <v>-1658307.05</v>
       </c>
     </row>
     <row r="167">
@@ -4610,7 +4610,7 @@
         </is>
       </c>
       <c r="E167" s="2" t="n">
-        <v>707099.0699999999</v>
+        <v>479110.27</v>
       </c>
     </row>
     <row r="168">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="E178" s="2" t="n">
-        <v>-1430318.25</v>
+        <v>-1658307.05</v>
       </c>
     </row>
     <row r="179">
@@ -4910,7 +4910,7 @@
         </is>
       </c>
       <c r="E179" s="2" t="n">
-        <v>707099.0699999999</v>
+        <v>479110.27</v>
       </c>
     </row>
     <row r="180">
@@ -4935,7 +4935,7 @@
         </is>
       </c>
       <c r="E180" s="2" t="n">
-        <v>707099.0699999999</v>
+        <v>479110.27</v>
       </c>
     </row>
     <row r="181">
@@ -7435,7 +7435,7 @@
         </is>
       </c>
       <c r="E280" s="2" t="n">
-        <v>-713853.33</v>
+        <v>-938367.77</v>
       </c>
     </row>
     <row r="281">
@@ -7460,7 +7460,7 @@
         </is>
       </c>
       <c r="E281" s="2" t="n">
-        <v>1137790.48</v>
+        <v>913276.04</v>
       </c>
     </row>
     <row r="282">
@@ -7510,7 +7510,7 @@
         </is>
       </c>
       <c r="E283" s="2" t="n">
-        <v>-0</v>
+        <v>-578969.26</v>
       </c>
     </row>
     <row r="284">
@@ -7535,7 +7535,7 @@
         </is>
       </c>
       <c r="E284" s="2" t="n">
-        <v>604858.9</v>
+        <v>25889.64</v>
       </c>
     </row>
     <row r="285">
@@ -7735,7 +7735,7 @@
         </is>
       </c>
       <c r="E292" s="2" t="n">
-        <v>-732753.33</v>
+        <v>-1536237.03</v>
       </c>
     </row>
     <row r="293">
@@ -7760,7 +7760,7 @@
         </is>
       </c>
       <c r="E293" s="2" t="n">
-        <v>1753749.38</v>
+        <v>950265.6800000001</v>
       </c>
     </row>
     <row r="294">
@@ -7785,7 +7785,7 @@
         </is>
       </c>
       <c r="E294" s="2" t="n">
-        <v>1753749.38</v>
+        <v>950265.6800000001</v>
       </c>
     </row>
     <row r="295">
@@ -7910,7 +7910,7 @@
         </is>
       </c>
       <c r="E299" s="2" t="n">
-        <v>-2590732.31</v>
+        <v>-2690482.31</v>
       </c>
     </row>
     <row r="300">
@@ -7935,7 +7935,7 @@
         </is>
       </c>
       <c r="E300" s="2" t="n">
-        <v>1524059.39</v>
+        <v>1424309.39</v>
       </c>
     </row>
     <row r="301">
@@ -8210,7 +8210,7 @@
         </is>
       </c>
       <c r="E311" s="2" t="n">
-        <v>-2590732.31</v>
+        <v>-2690482.31</v>
       </c>
     </row>
     <row r="312">
@@ -8235,7 +8235,7 @@
         </is>
       </c>
       <c r="E312" s="2" t="n">
-        <v>1524059.39</v>
+        <v>1424309.39</v>
       </c>
     </row>
     <row r="313">
@@ -8260,7 +8260,7 @@
         </is>
       </c>
       <c r="E313" s="2" t="n">
-        <v>1524059.39</v>
+        <v>1424309.39</v>
       </c>
     </row>
     <row r="314">
@@ -9435,7 +9435,7 @@
         </is>
       </c>
       <c r="E360" s="2" t="n">
-        <v>-2144384.8</v>
+        <v>-2126242.57</v>
       </c>
     </row>
     <row r="361">
@@ -9460,7 +9460,7 @@
         </is>
       </c>
       <c r="E361" s="2" t="n">
-        <v>1541369.65</v>
+        <v>1559511.88</v>
       </c>
     </row>
     <row r="362">
@@ -9735,7 +9735,7 @@
         </is>
       </c>
       <c r="E372" s="2" t="n">
-        <v>-2328659.8</v>
+        <v>-2310517.57</v>
       </c>
     </row>
     <row r="373">
@@ -9760,7 +9760,7 @@
         </is>
       </c>
       <c r="E373" s="2" t="n">
-        <v>1649594.65</v>
+        <v>1667736.88</v>
       </c>
     </row>
     <row r="374">
@@ -9785,7 +9785,7 @@
         </is>
       </c>
       <c r="E374" s="2" t="n">
-        <v>1649594.65</v>
+        <v>1667736.88</v>
       </c>
     </row>
     <row r="375">
@@ -10710,7 +10710,7 @@
         </is>
       </c>
       <c r="E411" s="2" t="n">
-        <v>-123338.12</v>
+        <v>-245290.26</v>
       </c>
     </row>
     <row r="412">
@@ -10735,7 +10735,7 @@
         </is>
       </c>
       <c r="E412" s="2" t="n">
-        <v>236506.36</v>
+        <v>114554.22</v>
       </c>
     </row>
     <row r="413">
@@ -10785,7 +10785,7 @@
         </is>
       </c>
       <c r="E414" s="2" t="n">
-        <v>-3177326.95</v>
+        <v>-3299279.09</v>
       </c>
     </row>
     <row r="415">
@@ -10810,7 +10810,7 @@
         </is>
       </c>
       <c r="E415" s="2" t="n">
-        <v>1727830.75</v>
+        <v>1605878.61</v>
       </c>
     </row>
     <row r="416">
@@ -10835,7 +10835,7 @@
         </is>
       </c>
       <c r="E416" s="2" t="n">
-        <v>1727830.75</v>
+        <v>1605878.61</v>
       </c>
     </row>
     <row r="417">
@@ -11435,7 +11435,7 @@
         </is>
       </c>
       <c r="E440" s="2" t="n">
-        <v>-2191516.17</v>
+        <v>-2256181.96</v>
       </c>
     </row>
     <row r="441">
@@ -11460,7 +11460,7 @@
         </is>
       </c>
       <c r="E441" s="2" t="n">
-        <v>1767594.02</v>
+        <v>1702928.23</v>
       </c>
     </row>
     <row r="442">
@@ -11510,7 +11510,7 @@
         </is>
       </c>
       <c r="E443" s="2" t="n">
-        <v>-28825.46</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="444">
@@ -11535,7 +11535,7 @@
         </is>
       </c>
       <c r="E444" s="2" t="n">
-        <v>16462.54</v>
+        <v>45288</v>
       </c>
     </row>
     <row r="445">
@@ -11585,7 +11585,7 @@
         </is>
       </c>
       <c r="E446" s="2" t="n">
-        <v>-86062.98</v>
+        <v>-189217.89</v>
       </c>
     </row>
     <row r="447">
@@ -11610,7 +11610,7 @@
         </is>
       </c>
       <c r="E447" s="2" t="n">
-        <v>303405.22</v>
+        <v>200250.31</v>
       </c>
     </row>
     <row r="448">
@@ -11660,7 +11660,7 @@
         </is>
       </c>
       <c r="E449" s="2" t="n">
-        <v>-368075.03</v>
+        <v>-176533.75</v>
       </c>
     </row>
     <row r="450">
@@ -11685,7 +11685,7 @@
         </is>
       </c>
       <c r="E450" s="2" t="n">
-        <v>1105119.47</v>
+        <v>1296660.75</v>
       </c>
     </row>
     <row r="451">
@@ -11735,7 +11735,7 @@
         </is>
       </c>
       <c r="E452" s="2" t="n">
-        <v>-2674479.64</v>
+        <v>-2773533.22</v>
       </c>
     </row>
     <row r="453">
@@ -11760,7 +11760,7 @@
         </is>
       </c>
       <c r="E453" s="2" t="n">
-        <v>3192581.25</v>
+        <v>3093527.67</v>
       </c>
     </row>
     <row r="454">
@@ -11785,7 +11785,7 @@
         </is>
       </c>
       <c r="E454" s="2" t="n">
-        <v>3192581.25</v>
+        <v>3093527.67</v>
       </c>
     </row>
     <row r="455">

</xml_diff>

<commit_message>
fix: LB financeiro por WS usa margem_projetos diretamente; merge J&J variants; display MB% consistente com LB
- real_mb_pct no detalhe_ws agora exibe MB% financeiro (real_lb_fin/real_rec) em vez de benchmark
- clientes.csv: alias J&J DO BRASIL INDUSTR → JOHNSON & JOHNSON para mesclar ambas as entradas SAP
- apuracao_engine.py: pré-normalização de nomes SAP antes do groupby (merge antes da agregação)
- remove entrada duplicada de ADCOS em clientes.csv
- regenera apuracao_q4_exportado.xlsx com valores consistentes

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/apuracao_q4_exportado.xlsx
+++ b/backend/apuracao_q4_exportado.xlsx
@@ -9910,7 +9910,7 @@
         </is>
       </c>
       <c r="E379" s="2" t="n">
-        <v>-5448861.23</v>
+        <v>-5557177.06</v>
       </c>
     </row>
     <row r="380">
@@ -9935,7 +9935,7 @@
         </is>
       </c>
       <c r="E380" s="2" t="n">
-        <v>3749070.41</v>
+        <v>3640754.58</v>
       </c>
     </row>
     <row r="381">
@@ -10210,7 +10210,7 @@
         </is>
       </c>
       <c r="E391" s="2" t="n">
-        <v>-7021944.84</v>
+        <v>-7130260.67</v>
       </c>
     </row>
     <row r="392">
@@ -10235,7 +10235,7 @@
         </is>
       </c>
       <c r="E392" s="2" t="n">
-        <v>4659143.13</v>
+        <v>4550827.3</v>
       </c>
     </row>
     <row r="393">
@@ -10710,7 +10710,7 @@
         </is>
       </c>
       <c r="E411" s="2" t="n">
-        <v>-245290.26</v>
+        <v>-103986.24</v>
       </c>
     </row>
     <row r="412">
@@ -10735,7 +10735,7 @@
         </is>
       </c>
       <c r="E412" s="2" t="n">
-        <v>114554.22</v>
+        <v>255858.24</v>
       </c>
     </row>
     <row r="413">
@@ -10785,7 +10785,7 @@
         </is>
       </c>
       <c r="E414" s="2" t="n">
-        <v>-3299279.09</v>
+        <v>-3157975.07</v>
       </c>
     </row>
     <row r="415">
@@ -10810,7 +10810,7 @@
         </is>
       </c>
       <c r="E415" s="2" t="n">
-        <v>1605878.61</v>
+        <v>1747182.63</v>
       </c>
     </row>
     <row r="416">
@@ -10835,7 +10835,7 @@
         </is>
       </c>
       <c r="E416" s="2" t="n">
-        <v>1605878.61</v>
+        <v>1747182.63</v>
       </c>
     </row>
     <row r="417">
@@ -11435,7 +11435,7 @@
         </is>
       </c>
       <c r="E440" s="2" t="n">
-        <v>-2256181.96</v>
+        <v>-2364497.79</v>
       </c>
     </row>
     <row r="441">
@@ -11460,7 +11460,7 @@
         </is>
       </c>
       <c r="E441" s="2" t="n">
-        <v>1702928.23</v>
+        <v>1594612.4</v>
       </c>
     </row>
     <row r="442">
@@ -11735,7 +11735,7 @@
         </is>
       </c>
       <c r="E452" s="2" t="n">
-        <v>-2773533.22</v>
+        <v>-2838565.26</v>
       </c>
     </row>
     <row r="453">
@@ -11760,7 +11760,7 @@
         </is>
       </c>
       <c r="E453" s="2" t="n">
-        <v>3093527.67</v>
+        <v>3028495.63</v>
       </c>
     </row>
     <row r="454">
@@ -11785,7 +11785,7 @@
         </is>
       </c>
       <c r="E454" s="2" t="n">
-        <v>3093527.67</v>
+        <v>3028495.63</v>
       </c>
     </row>
     <row r="455">

</xml_diff>

<commit_message>
fix: exclui projetos do time Hyper (empresa=Hyper/BR07) dos lookups de AE
Receita/margem do time Hyper estava sendo incorretamente atribuída
a AEs de outras verticais (ex: Vinicius/Health) por meio de clientes
compartilhados (ex: ODONTOPREV). Lookups _nh (non-Hyper) filtram
empresa Hyper/BR07 em rac_projetos e margem_projetos antes de calcular
proporção por WS. Diretores mantêm lookups completos (responsáveis
pela vertical inteira, incluindo time Hyper).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/apuracao_q4_exportado.xlsx
+++ b/backend/apuracao_q4_exportado.xlsx
@@ -7185,7 +7185,7 @@
         </is>
       </c>
       <c r="E270" s="2" t="n">
-        <v>604858.9</v>
+        <v>572779.74</v>
       </c>
     </row>
     <row r="271">
@@ -7410,7 +7410,7 @@
         </is>
       </c>
       <c r="E279" s="2" t="n">
-        <v>2486502.71</v>
+        <v>2454423.55</v>
       </c>
     </row>
     <row r="280">
@@ -11110,7 +11110,7 @@
         </is>
       </c>
       <c r="E427" s="2" t="n">
-        <v>389468.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="428">
@@ -11135,7 +11135,7 @@
         </is>
       </c>
       <c r="E428" s="2" t="n">
-        <v>-189217.89</v>
+        <v>0</v>
       </c>
     </row>
     <row r="429">
@@ -11160,7 +11160,7 @@
         </is>
       </c>
       <c r="E429" s="2" t="n">
-        <v>200250.31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="430">
@@ -11260,7 +11260,7 @@
         </is>
       </c>
       <c r="E433" s="2" t="n">
-        <v>5867060.89</v>
+        <v>5477592.69</v>
       </c>
     </row>
     <row r="434">
@@ -11285,7 +11285,7 @@
         </is>
       </c>
       <c r="E434" s="2" t="n">
-        <v>-2473314.55</v>
+        <v>-2284096.66</v>
       </c>
     </row>
     <row r="435">
@@ -11310,7 +11310,7 @@
         </is>
       </c>
       <c r="E435" s="2" t="n">
-        <v>3028495.63</v>
+        <v>2828245.32</v>
       </c>
     </row>
     <row r="436">

</xml_diff>

<commit_message>
fix: aplica benchmark MB% por WS no engine (Demais/Cloud/Dados/Hyper)
Projetos com custo_rateado=0 no SAP (ex: Dental Sorria) estavam gerando
MB%=100% na apuração. Alinha com a lógica de main.py que já aplicava
o benchmark antes de exibir na aba Margem por cliente.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/apuracao_q4_exportado.xlsx
+++ b/backend/apuracao_q4_exportado.xlsx
@@ -7210,7 +7210,7 @@
         </is>
       </c>
       <c r="E271" s="2" t="n">
-        <v>0</v>
+        <v>-16828.27</v>
       </c>
     </row>
     <row r="272">
@@ -7235,7 +7235,7 @@
         </is>
       </c>
       <c r="E272" s="2" t="n">
-        <v>25889.64</v>
+        <v>9061.370000000001</v>
       </c>
     </row>
     <row r="273">
@@ -7435,7 +7435,7 @@
         </is>
       </c>
       <c r="E280" s="2" t="n">
-        <v>-732753.33</v>
+        <v>-749581.6</v>
       </c>
     </row>
     <row r="281">
@@ -7460,7 +7460,7 @@
         </is>
       </c>
       <c r="E281" s="2" t="n">
-        <v>950265.6800000001</v>
+        <v>933437.41</v>
       </c>
     </row>
     <row r="282">
@@ -10310,7 +10310,7 @@
         </is>
       </c>
       <c r="E395" s="2" t="n">
-        <v>-123338.12</v>
+        <v>-238893.71</v>
       </c>
     </row>
     <row r="396">
@@ -10335,7 +10335,7 @@
         </is>
       </c>
       <c r="E396" s="2" t="n">
-        <v>255858.24</v>
+        <v>140302.65</v>
       </c>
     </row>
     <row r="397">
@@ -10385,7 +10385,7 @@
         </is>
       </c>
       <c r="E398" s="2" t="n">
-        <v>-3177326.95</v>
+        <v>-3292882.54</v>
       </c>
     </row>
     <row r="399">
@@ -10410,7 +10410,7 @@
         </is>
       </c>
       <c r="E399" s="2" t="n">
-        <v>1747182.63</v>
+        <v>1631627.04</v>
       </c>
     </row>
     <row r="400">
@@ -11060,7 +11060,7 @@
         </is>
       </c>
       <c r="E425" s="2" t="n">
-        <v>0</v>
+        <v>-29437.2</v>
       </c>
     </row>
     <row r="426">
@@ -11085,7 +11085,7 @@
         </is>
       </c>
       <c r="E426" s="2" t="n">
-        <v>45288</v>
+        <v>15850.8</v>
       </c>
     </row>
     <row r="427">
@@ -11210,7 +11210,7 @@
         </is>
       </c>
       <c r="E431" s="2" t="n">
-        <v>-120763.96</v>
+        <v>-914905.5699999999</v>
       </c>
     </row>
     <row r="432">
@@ -11235,7 +11235,7 @@
         </is>
       </c>
       <c r="E432" s="2" t="n">
-        <v>1296660.75</v>
+        <v>502519.14</v>
       </c>
     </row>
     <row r="433">
@@ -11285,7 +11285,7 @@
         </is>
       </c>
       <c r="E434" s="2" t="n">
-        <v>-2284096.66</v>
+        <v>-3107675.47</v>
       </c>
     </row>
     <row r="435">
@@ -11310,7 +11310,7 @@
         </is>
       </c>
       <c r="E435" s="2" t="n">
-        <v>2828245.32</v>
+        <v>2004666.51</v>
       </c>
     </row>
     <row r="436">

</xml_diff>

<commit_message>
chore: atualiza apuracao_q4_exportado com correções de lb/custo/benchmark
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/apuracao_q4_exportado.xlsx
+++ b/backend/apuracao_q4_exportado.xlsx
@@ -7210,7 +7210,7 @@
         </is>
       </c>
       <c r="E271" s="2" t="n">
-        <v>-16828.27</v>
+        <v>-372306.83</v>
       </c>
     </row>
     <row r="272">
@@ -7235,7 +7235,7 @@
         </is>
       </c>
       <c r="E272" s="2" t="n">
-        <v>9061.370000000001</v>
+        <v>200472.91</v>
       </c>
     </row>
     <row r="273">
@@ -7435,7 +7435,7 @@
         </is>
       </c>
       <c r="E280" s="2" t="n">
-        <v>-749581.6</v>
+        <v>-1105060.16</v>
       </c>
     </row>
     <row r="281">
@@ -7460,7 +7460,7 @@
         </is>
       </c>
       <c r="E281" s="2" t="n">
-        <v>933437.41</v>
+        <v>1124848.95</v>
       </c>
     </row>
     <row r="282">
@@ -10310,7 +10310,7 @@
         </is>
       </c>
       <c r="E395" s="2" t="n">
-        <v>-238893.71</v>
+        <v>-226702.02</v>
       </c>
     </row>
     <row r="396">
@@ -10335,7 +10335,7 @@
         </is>
       </c>
       <c r="E396" s="2" t="n">
-        <v>140302.65</v>
+        <v>133142.46</v>
       </c>
     </row>
     <row r="397">
@@ -10385,7 +10385,7 @@
         </is>
       </c>
       <c r="E398" s="2" t="n">
-        <v>-3292882.54</v>
+        <v>-3280690.86</v>
       </c>
     </row>
     <row r="399">
@@ -10410,7 +10410,7 @@
         </is>
       </c>
       <c r="E399" s="2" t="n">
-        <v>1631627.04</v>
+        <v>1624466.84</v>
       </c>
     </row>
     <row r="400">
@@ -11210,7 +11210,7 @@
         </is>
       </c>
       <c r="E431" s="2" t="n">
-        <v>-914905.5699999999</v>
+        <v>-928112.54</v>
       </c>
     </row>
     <row r="432">
@@ -11235,7 +11235,7 @@
         </is>
       </c>
       <c r="E432" s="2" t="n">
-        <v>502519.14</v>
+        <v>545081.96</v>
       </c>
     </row>
     <row r="433">
@@ -11285,7 +11285,7 @@
         </is>
       </c>
       <c r="E434" s="2" t="n">
-        <v>-3107675.47</v>
+        <v>-3322047.53</v>
       </c>
     </row>
     <row r="435">
@@ -11310,7 +11310,7 @@
         </is>
       </c>
       <c r="E435" s="2" t="n">
-        <v>2004666.51</v>
+        <v>2155545.16</v>
       </c>
     </row>
     <row r="436">

</xml_diff>

<commit_message>
feat: engine diretores usa escopo por PEP (espelha MargemTab)
- Troca loops de clientes por loop pep-based em calc_bonus_diretor
- LB% e margem dos diretores agora batem exatamente com a aba Margem por Cliente
- Meta MC dos diretores: valor absoluto R$ (metas_mc_dir.csv) com gatilho 85%
- Novos clientes Finance: TRANSUNION, YELUM SEGUROS; Karina → Others no pep_vertical
- Excel apuracao_q4_exportado regenerado

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/apuracao_q4_exportado.xlsx
+++ b/backend/apuracao_q4_exportado.xlsx
@@ -433,7 +433,7 @@
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5177271.64</v>
+        <v>12190846.81</v>
       </c>
     </row>
     <row r="6">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>-3444306.98</v>
+        <v>-8914030.9</v>
       </c>
     </row>
     <row r="7">
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1732964.66</v>
+        <v>3276815.91</v>
       </c>
     </row>
     <row r="8">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>578052.61</v>
+        <v>638826.13</v>
       </c>
     </row>
     <row r="12">
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-375734.2</v>
+        <v>-415236.98</v>
       </c>
     </row>
     <row r="13">
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>202318.41</v>
+        <v>223589.15</v>
       </c>
     </row>
     <row r="14">
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>1152892.68</v>
+        <v>2772052.34</v>
       </c>
     </row>
     <row r="15">
@@ -810,7 +810,7 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>-726322.39</v>
+        <v>-1746392.97</v>
       </c>
     </row>
     <row r="16">
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>426570.29</v>
+        <v>1025659.37</v>
       </c>
     </row>
     <row r="17">
@@ -860,7 +860,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>6908216.93</v>
+        <v>15601725.28</v>
       </c>
     </row>
     <row r="18">
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>-4546363.57</v>
+        <v>-11075660.85</v>
       </c>
     </row>
     <row r="19">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>2361853.36</v>
+        <v>4526064.43</v>
       </c>
     </row>
     <row r="20">
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0</v>
+        <v>188722.96</v>
       </c>
     </row>
     <row r="26">
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>-0</v>
+        <v>-124557.15</v>
       </c>
     </row>
     <row r="27">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0</v>
+        <v>64165.81</v>
       </c>
     </row>
     <row r="28">
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>5150089.72</v>
+        <v>5882054.79</v>
       </c>
     </row>
     <row r="29">
@@ -1160,7 +1160,7 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>-2197418.88</v>
+        <v>-3184656.42</v>
       </c>
     </row>
     <row r="30">
@@ -1185,7 +1185,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>2952670.84</v>
+        <v>2697398.37</v>
       </c>
     </row>
     <row r="31">
@@ -1210,7 +1210,7 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>604858.9</v>
+        <v>902579.42</v>
       </c>
     </row>
     <row r="32">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>-393158.29</v>
+        <v>-586676.62</v>
       </c>
     </row>
     <row r="33">
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>211700.61</v>
+        <v>315902.8</v>
       </c>
     </row>
     <row r="34">
@@ -1285,7 +1285,7 @@
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>402406.65</v>
+        <v>403147.47</v>
       </c>
     </row>
     <row r="35">
@@ -1310,7 +1310,7 @@
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>-261564.32</v>
+        <v>-262045.86</v>
       </c>
     </row>
     <row r="36">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>140842.33</v>
+        <v>141101.61</v>
       </c>
     </row>
     <row r="37">
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>127180.22</v>
+        <v>214987.32</v>
       </c>
     </row>
     <row r="38">
@@ -1385,7 +1385,7 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>-80123.53999999999</v>
+        <v>-135442.01</v>
       </c>
     </row>
     <row r="39">
@@ -1410,7 +1410,7 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>47056.68</v>
+        <v>79545.31</v>
       </c>
     </row>
     <row r="40">
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>6284535.49</v>
+        <v>7591491.96</v>
       </c>
     </row>
     <row r="41">
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>-2932265.03</v>
+        <v>-4293378.06</v>
       </c>
     </row>
     <row r="42">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>3352270.46</v>
+        <v>3298113.9</v>
       </c>
     </row>
     <row r="43">
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="E142" s="2" t="n">
-        <v>-1426517.06</v>
+        <v>-1446757.06</v>
       </c>
     </row>
     <row r="143">
@@ -4010,7 +4010,7 @@
         </is>
       </c>
       <c r="E143" s="2" t="n">
-        <v>1171838.36</v>
+        <v>1151598.36</v>
       </c>
     </row>
     <row r="144">
@@ -4285,7 +4285,7 @@
         </is>
       </c>
       <c r="E154" s="2" t="n">
-        <v>-1426517.06</v>
+        <v>-1446757.06</v>
       </c>
     </row>
     <row r="155">
@@ -4310,7 +4310,7 @@
         </is>
       </c>
       <c r="E155" s="2" t="n">
-        <v>1171838.36</v>
+        <v>1151598.36</v>
       </c>
     </row>
     <row r="156">
@@ -4435,7 +4435,7 @@
         </is>
       </c>
       <c r="E160" s="2" t="n">
-        <v>-1430318.25</v>
+        <v>-1681883.3</v>
       </c>
     </row>
     <row r="161">
@@ -4460,7 +4460,7 @@
         </is>
       </c>
       <c r="E161" s="2" t="n">
-        <v>479110.27</v>
+        <v>227545.22</v>
       </c>
     </row>
     <row r="162">
@@ -4735,7 +4735,7 @@
         </is>
       </c>
       <c r="E172" s="2" t="n">
-        <v>-1430318.25</v>
+        <v>-1681883.3</v>
       </c>
     </row>
     <row r="173">
@@ -4760,7 +4760,7 @@
         </is>
       </c>
       <c r="E173" s="2" t="n">
-        <v>479110.27</v>
+        <v>227545.22</v>
       </c>
     </row>
     <row r="174">
@@ -7035,7 +7035,7 @@
         </is>
       </c>
       <c r="E264" s="2" t="n">
-        <v>0</v>
+        <v>166549.02</v>
       </c>
     </row>
     <row r="265">
@@ -7060,7 +7060,7 @@
         </is>
       </c>
       <c r="E265" s="2" t="n">
-        <v>0</v>
+        <v>-109922.35</v>
       </c>
     </row>
     <row r="266">
@@ -7085,7 +7085,7 @@
         </is>
       </c>
       <c r="E266" s="2" t="n">
-        <v>0</v>
+        <v>56626.67</v>
       </c>
     </row>
     <row r="267">
@@ -7110,7 +7110,7 @@
         </is>
       </c>
       <c r="E267" s="2" t="n">
-        <v>1851643.81</v>
+        <v>2180205.61</v>
       </c>
     </row>
     <row r="268">
@@ -7135,7 +7135,7 @@
         </is>
       </c>
       <c r="E268" s="2" t="n">
-        <v>-713853.33</v>
+        <v>-650050.16</v>
       </c>
     </row>
     <row r="269">
@@ -7160,7 +7160,7 @@
         </is>
       </c>
       <c r="E269" s="2" t="n">
-        <v>913276.04</v>
+        <v>746305.74</v>
       </c>
     </row>
     <row r="270">
@@ -7185,7 +7185,7 @@
         </is>
       </c>
       <c r="E270" s="2" t="n">
-        <v>572779.74</v>
+        <v>77668.92</v>
       </c>
     </row>
     <row r="271">
@@ -7210,7 +7210,7 @@
         </is>
       </c>
       <c r="E271" s="2" t="n">
-        <v>-372306.83</v>
+        <v>-50484.8</v>
       </c>
     </row>
     <row r="272">
@@ -7235,7 +7235,7 @@
         </is>
       </c>
       <c r="E272" s="2" t="n">
-        <v>200472.91</v>
+        <v>27184.12</v>
       </c>
     </row>
     <row r="273">
@@ -7435,7 +7435,7 @@
         </is>
       </c>
       <c r="E280" s="2" t="n">
-        <v>-1105060.16</v>
+        <v>-829357.3100000001</v>
       </c>
     </row>
     <row r="281">
@@ -7460,7 +7460,7 @@
         </is>
       </c>
       <c r="E281" s="2" t="n">
-        <v>1124848.95</v>
+        <v>841216.53</v>
       </c>
     </row>
     <row r="282">
@@ -8010,7 +8010,7 @@
         </is>
       </c>
       <c r="E303" s="2" t="n">
-        <v>11126186.43</v>
+        <v>11539673.15</v>
       </c>
     </row>
     <row r="304">
@@ -8035,7 +8035,7 @@
         </is>
       </c>
       <c r="E304" s="2" t="n">
-        <v>-6619865.57</v>
+        <v>-7425141.36</v>
       </c>
     </row>
     <row r="305">
@@ -8060,7 +8060,7 @@
         </is>
       </c>
       <c r="E305" s="2" t="n">
-        <v>4506320.86</v>
+        <v>4114531.79</v>
       </c>
     </row>
     <row r="306">
@@ -8160,7 +8160,7 @@
         </is>
       </c>
       <c r="E309" s="2" t="n">
-        <v>0</v>
+        <v>62118.66</v>
       </c>
     </row>
     <row r="310">
@@ -8185,7 +8185,7 @@
         </is>
       </c>
       <c r="E310" s="2" t="n">
-        <v>-0</v>
+        <v>-40377.13</v>
       </c>
     </row>
     <row r="311">
@@ -8210,7 +8210,7 @@
         </is>
       </c>
       <c r="E311" s="2" t="n">
-        <v>0</v>
+        <v>21741.53</v>
       </c>
     </row>
     <row r="312">
@@ -8235,7 +8235,7 @@
         </is>
       </c>
       <c r="E312" s="2" t="n">
-        <v>0</v>
+        <v>-188859.67</v>
       </c>
     </row>
     <row r="313">
@@ -8260,7 +8260,7 @@
         </is>
       </c>
       <c r="E313" s="2" t="n">
-        <v>-0</v>
+        <v>188859.67</v>
       </c>
     </row>
     <row r="314">
@@ -8310,7 +8310,7 @@
         </is>
       </c>
       <c r="E315" s="2" t="n">
-        <v>11126186.43</v>
+        <v>11412932.14</v>
       </c>
     </row>
     <row r="316">
@@ -8335,7 +8335,7 @@
         </is>
       </c>
       <c r="E316" s="2" t="n">
-        <v>-6619865.57</v>
+        <v>-7276658.82</v>
       </c>
     </row>
     <row r="317">
@@ -8360,7 +8360,7 @@
         </is>
       </c>
       <c r="E317" s="2" t="n">
-        <v>4506320.86</v>
+        <v>4136273.32</v>
       </c>
     </row>
     <row r="318">
@@ -8585,7 +8585,7 @@
         </is>
       </c>
       <c r="E326" s="2" t="n">
-        <v>2458912.71</v>
+        <v>3822498.48</v>
       </c>
     </row>
     <row r="327">
@@ -8610,7 +8610,7 @@
         </is>
       </c>
       <c r="E327" s="2" t="n">
-        <v>-1349591.15</v>
+        <v>-1827759.16</v>
       </c>
     </row>
     <row r="328">
@@ -8635,7 +8635,7 @@
         </is>
       </c>
       <c r="E328" s="2" t="n">
-        <v>1109321.56</v>
+        <v>2001739</v>
       </c>
     </row>
     <row r="329">
@@ -8810,7 +8810,7 @@
         </is>
       </c>
       <c r="E335" s="2" t="n">
-        <v>0</v>
+        <v>440669.63</v>
       </c>
     </row>
     <row r="336">
@@ -8835,7 +8835,7 @@
         </is>
       </c>
       <c r="E336" s="2" t="n">
-        <v>0</v>
+        <v>-277621.87</v>
       </c>
     </row>
     <row r="337">
@@ -8860,7 +8860,7 @@
         </is>
       </c>
       <c r="E337" s="2" t="n">
-        <v>0</v>
+        <v>163047.76</v>
       </c>
     </row>
     <row r="338">
@@ -8885,7 +8885,7 @@
         </is>
       </c>
       <c r="E338" s="2" t="n">
-        <v>2458912.71</v>
+        <v>4263168.11</v>
       </c>
     </row>
     <row r="339">
@@ -8910,7 +8910,7 @@
         </is>
       </c>
       <c r="E339" s="2" t="n">
-        <v>-1349591.15</v>
+        <v>-2105381.03</v>
       </c>
     </row>
     <row r="340">
@@ -8935,7 +8935,7 @@
         </is>
       </c>
       <c r="E340" s="2" t="n">
-        <v>1109321.56</v>
+        <v>2164786.77</v>
       </c>
     </row>
     <row r="341">
@@ -9060,7 +9060,7 @@
         </is>
       </c>
       <c r="E345" s="2" t="n">
-        <v>-2144384.8</v>
+        <v>-2145446.18</v>
       </c>
     </row>
     <row r="346">
@@ -9085,7 +9085,7 @@
         </is>
       </c>
       <c r="E346" s="2" t="n">
-        <v>1559511.88</v>
+        <v>1558450.5</v>
       </c>
     </row>
     <row r="347">
@@ -9360,7 +9360,7 @@
         </is>
       </c>
       <c r="E357" s="2" t="n">
-        <v>-2328659.8</v>
+        <v>-2329721.18</v>
       </c>
     </row>
     <row r="358">
@@ -9385,7 +9385,7 @@
         </is>
       </c>
       <c r="E358" s="2" t="n">
-        <v>1667736.88</v>
+        <v>1666675.5</v>
       </c>
     </row>
     <row r="359">
@@ -9485,7 +9485,7 @@
         </is>
       </c>
       <c r="E362" s="2" t="n">
-        <v>9197931.640000001</v>
+        <v>10179598.96</v>
       </c>
     </row>
     <row r="363">
@@ -9510,7 +9510,7 @@
         </is>
       </c>
       <c r="E363" s="2" t="n">
-        <v>-5557177.06</v>
+        <v>-6005376.54</v>
       </c>
     </row>
     <row r="364">
@@ -9535,7 +9535,7 @@
         </is>
       </c>
       <c r="E364" s="2" t="n">
-        <v>3640754.58</v>
+        <v>4174222.42</v>
       </c>
     </row>
     <row r="365">
@@ -9635,7 +9635,7 @@
         </is>
       </c>
       <c r="E368" s="2" t="n">
-        <v>389468.2</v>
+        <v>426454.36</v>
       </c>
     </row>
     <row r="369">
@@ -9660,7 +9660,7 @@
         </is>
       </c>
       <c r="E369" s="2" t="n">
-        <v>-253154.33</v>
+        <v>-277195.33</v>
       </c>
     </row>
     <row r="370">
@@ -9685,7 +9685,7 @@
         </is>
       </c>
       <c r="E370" s="2" t="n">
-        <v>136313.87</v>
+        <v>149259.03</v>
       </c>
     </row>
     <row r="371">
@@ -9710,7 +9710,7 @@
         </is>
       </c>
       <c r="E371" s="2" t="n">
-        <v>2048400.13</v>
+        <v>2744820.5</v>
       </c>
     </row>
     <row r="372">
@@ -9735,7 +9735,7 @@
         </is>
       </c>
       <c r="E372" s="2" t="n">
-        <v>-1290492.08</v>
+        <v>-1729236.92</v>
       </c>
     </row>
     <row r="373">
@@ -9760,7 +9760,7 @@
         </is>
       </c>
       <c r="E373" s="2" t="n">
-        <v>757908.05</v>
+        <v>1015583.58</v>
       </c>
     </row>
     <row r="374">
@@ -9785,7 +9785,7 @@
         </is>
       </c>
       <c r="E374" s="2" t="n">
-        <v>11681087.97</v>
+        <v>13396161.82</v>
       </c>
     </row>
     <row r="375">
@@ -9810,7 +9810,7 @@
         </is>
       </c>
       <c r="E375" s="2" t="n">
-        <v>-7130260.67</v>
+        <v>-8041245.99</v>
       </c>
     </row>
     <row r="376">
@@ -9835,7 +9835,7 @@
         </is>
       </c>
       <c r="E376" s="2" t="n">
-        <v>4550827.3</v>
+        <v>5354915.83</v>
       </c>
     </row>
     <row r="377">
@@ -10085,7 +10085,7 @@
         </is>
       </c>
       <c r="E386" s="2" t="n">
-        <v>-3053988.83</v>
+        <v>-3292940.41</v>
       </c>
     </row>
     <row r="387">
@@ -10110,7 +10110,7 @@
         </is>
       </c>
       <c r="E387" s="2" t="n">
-        <v>1491324.39</v>
+        <v>1252372.81</v>
       </c>
     </row>
     <row r="388">
@@ -10385,7 +10385,7 @@
         </is>
       </c>
       <c r="E398" s="2" t="n">
-        <v>-3280690.86</v>
+        <v>-3519642.43</v>
       </c>
     </row>
     <row r="399">
@@ -10410,7 +10410,7 @@
         </is>
       </c>
       <c r="E399" s="2" t="n">
-        <v>1624466.84</v>
+        <v>1385515.27</v>
       </c>
     </row>
     <row r="400">
@@ -10985,7 +10985,7 @@
         </is>
       </c>
       <c r="E422" s="2" t="n">
-        <v>-2364497.79</v>
+        <v>-2401132.25</v>
       </c>
     </row>
     <row r="423">
@@ -11010,7 +11010,7 @@
         </is>
       </c>
       <c r="E423" s="2" t="n">
-        <v>1594612.4</v>
+        <v>1557977.94</v>
       </c>
     </row>
     <row r="424">
@@ -11285,7 +11285,7 @@
         </is>
       </c>
       <c r="E434" s="2" t="n">
-        <v>-3322047.53</v>
+        <v>-3358681.99</v>
       </c>
     </row>
     <row r="435">
@@ -11310,7 +11310,7 @@
         </is>
       </c>
       <c r="E435" s="2" t="n">
-        <v>2155545.16</v>
+        <v>2118910.7</v>
       </c>
     </row>
     <row r="436">
@@ -11410,7 +11410,7 @@
         </is>
       </c>
       <c r="E439" s="2" t="n">
-        <v>13825143.05</v>
+        <v>16043084.54</v>
       </c>
     </row>
     <row r="440">
@@ -11435,7 +11435,7 @@
         </is>
       </c>
       <c r="E440" s="2" t="n">
-        <v>-8779281.42</v>
+        <v>-9487141.949999999</v>
       </c>
     </row>
     <row r="441">
@@ -11460,7 +11460,7 @@
         </is>
       </c>
       <c r="E441" s="2" t="n">
-        <v>5045861.63</v>
+        <v>6555942.59</v>
       </c>
     </row>
     <row r="442">
@@ -11560,7 +11560,7 @@
         </is>
       </c>
       <c r="E445" s="2" t="n">
-        <v>0</v>
+        <v>387515.97</v>
       </c>
     </row>
     <row r="446">
@@ -11585,7 +11585,7 @@
         </is>
       </c>
       <c r="E446" s="2" t="n">
-        <v>-0</v>
+        <v>-251885.38</v>
       </c>
     </row>
     <row r="447">
@@ -11610,7 +11610,7 @@
         </is>
       </c>
       <c r="E447" s="2" t="n">
-        <v>0</v>
+        <v>135630.59</v>
       </c>
     </row>
     <row r="448">
@@ -11635,7 +11635,7 @@
         </is>
       </c>
       <c r="E448" s="2" t="n">
-        <v>684750</v>
+        <v>809410.62</v>
       </c>
     </row>
     <row r="449">
@@ -11660,7 +11660,7 @@
         </is>
       </c>
       <c r="E449" s="2" t="n">
-        <v>-431392.5</v>
+        <v>-509928.69</v>
       </c>
     </row>
     <row r="450">
@@ -11685,7 +11685,7 @@
         </is>
       </c>
       <c r="E450" s="2" t="n">
-        <v>253357.5</v>
+        <v>299481.93</v>
       </c>
     </row>
     <row r="451">
@@ -11710,7 +11710,7 @@
         </is>
       </c>
       <c r="E451" s="2" t="n">
-        <v>14509893.05</v>
+        <v>17240011.13</v>
       </c>
     </row>
     <row r="452">
@@ -11735,7 +11735,7 @@
         </is>
       </c>
       <c r="E452" s="2" t="n">
-        <v>-9210673.92</v>
+        <v>-10248956.02</v>
       </c>
     </row>
     <row r="453">
@@ -11760,7 +11760,7 @@
         </is>
       </c>
       <c r="E453" s="2" t="n">
-        <v>5299219.13</v>
+        <v>6991055.109999999</v>
       </c>
     </row>
     <row r="454">

</xml_diff>

<commit_message>
fix: MB% do breakdown WS bate com MB% da Carteira de Clientes
- Remove override de real_lb_ws por benchmark no detalhe_ws_dir
- realized_lb_ws_dir já usa SAP margem (benchmark aplicado em _load_all)
- realized_rec_ws_dir agora usa SAP receita (não RAC-escalado)
- Delta entre Receita por WS e Carteira de Clientes: 0.00pp em todos os diretores

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/apuracao_q4_exportado.xlsx
+++ b/backend/apuracao_q4_exportado.xlsx
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>188722.96</v>
+        <v>166549.02</v>
       </c>
     </row>
     <row r="26">
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>-124557.15</v>
+        <v>-109922.35</v>
       </c>
     </row>
     <row r="27">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>64165.81</v>
+        <v>56626.67</v>
       </c>
     </row>
     <row r="28">
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>5882054.79</v>
+        <v>5796717.21</v>
       </c>
     </row>
     <row r="29">
@@ -1160,7 +1160,7 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>-3184656.42</v>
+        <v>-3099318.84</v>
       </c>
     </row>
     <row r="30">
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>214987.32</v>
+        <v>322498.84</v>
       </c>
     </row>
     <row r="38">
@@ -1385,7 +1385,7 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>-135442.01</v>
+        <v>-203174.27</v>
       </c>
     </row>
     <row r="39">
@@ -1410,7 +1410,7 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>79545.31</v>
+        <v>119324.57</v>
       </c>
     </row>
     <row r="40">
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>-4293378.06</v>
+        <v>-4261137.94</v>
       </c>
     </row>
     <row r="42">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>3298113.9</v>
+        <v>3330354.02</v>
       </c>
     </row>
     <row r="43">
@@ -8010,7 +8010,7 @@
         </is>
       </c>
       <c r="E303" s="2" t="n">
-        <v>11539673.15</v>
+        <v>11350813.48</v>
       </c>
     </row>
     <row r="304">
@@ -8035,7 +8035,7 @@
         </is>
       </c>
       <c r="E304" s="2" t="n">
-        <v>-7425141.36</v>
+        <v>-7236281.69</v>
       </c>
     </row>
     <row r="305">
@@ -8235,7 +8235,7 @@
         </is>
       </c>
       <c r="E312" s="2" t="n">
-        <v>-188859.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="313">
@@ -8260,7 +8260,7 @@
         </is>
       </c>
       <c r="E313" s="2" t="n">
-        <v>188859.67</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="314">
@@ -9485,7 +9485,7 @@
         </is>
       </c>
       <c r="E362" s="2" t="n">
-        <v>10179598.96</v>
+        <v>10171510.54</v>
       </c>
     </row>
     <row r="363">
@@ -9510,7 +9510,7 @@
         </is>
       </c>
       <c r="E363" s="2" t="n">
-        <v>-6005376.54</v>
+        <v>-5997288.12</v>
       </c>
     </row>
     <row r="364">
@@ -9660,7 +9660,7 @@
         </is>
       </c>
       <c r="E369" s="2" t="n">
-        <v>-277195.33</v>
+        <v>-288647.12</v>
       </c>
     </row>
     <row r="370">
@@ -9685,7 +9685,7 @@
         </is>
       </c>
       <c r="E370" s="2" t="n">
-        <v>149259.03</v>
+        <v>137807.24</v>
       </c>
     </row>
     <row r="371">
@@ -9710,7 +9710,7 @@
         </is>
       </c>
       <c r="E371" s="2" t="n">
-        <v>2744820.5</v>
+        <v>2752908.92</v>
       </c>
     </row>
     <row r="372">
@@ -9735,7 +9735,7 @@
         </is>
       </c>
       <c r="E372" s="2" t="n">
-        <v>-1729236.92</v>
+        <v>-1756260.62</v>
       </c>
     </row>
     <row r="373">
@@ -9760,7 +9760,7 @@
         </is>
       </c>
       <c r="E373" s="2" t="n">
-        <v>1015583.58</v>
+        <v>996648.3</v>
       </c>
     </row>
     <row r="374">
@@ -9810,7 +9810,7 @@
         </is>
       </c>
       <c r="E375" s="2" t="n">
-        <v>-8041245.99</v>
+        <v>-8071633.06</v>
       </c>
     </row>
     <row r="376">
@@ -9835,7 +9835,7 @@
         </is>
       </c>
       <c r="E376" s="2" t="n">
-        <v>5354915.83</v>
+        <v>5324528.76</v>
       </c>
     </row>
     <row r="377">
@@ -11410,7 +11410,7 @@
         </is>
       </c>
       <c r="E439" s="2" t="n">
-        <v>16043084.54</v>
+        <v>16026575.21</v>
       </c>
     </row>
     <row r="440">
@@ -11435,7 +11435,7 @@
         </is>
       </c>
       <c r="E440" s="2" t="n">
-        <v>-9487141.949999999</v>
+        <v>-9470632.619999999</v>
       </c>
     </row>
     <row r="441">
@@ -11635,7 +11635,7 @@
         </is>
       </c>
       <c r="E448" s="2" t="n">
-        <v>809410.62</v>
+        <v>825919.95</v>
       </c>
     </row>
     <row r="449">
@@ -11660,7 +11660,7 @@
         </is>
       </c>
       <c r="E449" s="2" t="n">
-        <v>-509928.69</v>
+        <v>-854886.62</v>
       </c>
     </row>
     <row r="450">
@@ -11685,7 +11685,7 @@
         </is>
       </c>
       <c r="E450" s="2" t="n">
-        <v>299481.93</v>
+        <v>-28966.67</v>
       </c>
     </row>
     <row r="451">
@@ -11735,7 +11735,7 @@
         </is>
       </c>
       <c r="E452" s="2" t="n">
-        <v>-10248956.02</v>
+        <v>-10577404.62</v>
       </c>
     </row>
     <row r="453">
@@ -11760,7 +11760,7 @@
         </is>
       </c>
       <c r="E453" s="2" t="n">
-        <v>6991055.109999999</v>
+        <v>6662606.51</v>
       </c>
     </row>
     <row r="454">

</xml_diff>

<commit_message>
Move arquivos legados e scripts one-shot para backend/old/
CSVs consolidados (rac_projetos, margem_projetos, sap_agg, razao_agg,
tcv_realizado, q3_realizados_gm) substituidos por projetos.csv,
financeiro.csv e realizados_manual.csv.

Scripts de debug/analise pontuais (check_*, debug_*, gen_*, extract_*,
fix_*, fill_*, restore_*, update_*) preservados em old/ para referencia.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/apuracao_q4_exportado.xlsx
+++ b/backend/apuracao_q4_exportado.xlsx
@@ -433,7 +433,7 @@
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>3758108.11</v>
+        <v>3678409.51</v>
       </c>
     </row>
     <row r="10">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.7444</v>
+        <v>0.7392</v>
       </c>
     </row>
     <row r="11">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>29.01</v>
+        <v>28.78</v>
       </c>
     </row>
     <row r="12">
@@ -810,7 +810,7 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>12190846.81</v>
+        <v>12105554.24</v>
       </c>
     </row>
     <row r="16">
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>-8914030.9</v>
+        <v>-8858626.9</v>
       </c>
     </row>
     <row r="17">
@@ -860,7 +860,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>3276815.91</v>
+        <v>3246927.34</v>
       </c>
     </row>
     <row r="18">
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>638826.13</v>
+        <v>73917.02</v>
       </c>
     </row>
     <row r="22">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>-415236.98</v>
+        <v>-48046.06</v>
       </c>
     </row>
     <row r="23">
@@ -1010,7 +1010,7 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>223589.15</v>
+        <v>25870.96</v>
       </c>
     </row>
     <row r="24">
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>2772052.34</v>
+        <v>2819287.29</v>
       </c>
     </row>
     <row r="25">
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>-1746392.97</v>
+        <v>-1776150.99</v>
       </c>
     </row>
     <row r="26">
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>1025659.37</v>
+        <v>1043136.3</v>
       </c>
     </row>
     <row r="27">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>15601725.28</v>
+        <v>14998758.55</v>
       </c>
     </row>
     <row r="28">
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>-11075660.85</v>
+        <v>-10682823.95</v>
       </c>
     </row>
     <row r="29">
@@ -1160,7 +1160,7 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>4526064.43</v>
+        <v>4315934.6</v>
       </c>
     </row>
     <row r="30">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>2956681.62</v>
+        <v>2900236.83</v>
       </c>
     </row>
     <row r="43">
@@ -1510,7 +1510,7 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.9147999999999999</v>
+        <v>0.9069</v>
       </c>
     </row>
     <row r="44">
@@ -1535,7 +1535,7 @@
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>43.87</v>
+        <v>44.32</v>
       </c>
     </row>
     <row r="45">
@@ -1785,7 +1785,7 @@
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>403147.47</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -1810,7 +1810,7 @@
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>-262045.86</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="56">
@@ -1835,7 +1835,7 @@
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>141101.61</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -1860,7 +1860,7 @@
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>322498.84</v>
+        <v>372961.84</v>
       </c>
     </row>
     <row r="58">
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>-203174.27</v>
+        <v>-234965.96</v>
       </c>
     </row>
     <row r="59">
@@ -1910,7 +1910,7 @@
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>119324.57</v>
+        <v>137995.88</v>
       </c>
     </row>
     <row r="60">
@@ -1935,7 +1935,7 @@
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>7591491.96</v>
+        <v>7238807.49</v>
       </c>
     </row>
     <row r="61">
@@ -1960,7 +1960,7 @@
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>-4261137.94</v>
+        <v>-4030883.77</v>
       </c>
     </row>
     <row r="62">
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>3330354.02</v>
+        <v>3207923.72</v>
       </c>
     </row>
     <row r="63">
@@ -5415,7 +5415,7 @@
         </is>
       </c>
       <c r="E200" s="2" t="n">
-        <v>4465112.66</v>
+        <v>5025921</v>
       </c>
     </row>
     <row r="201">
@@ -5440,7 +5440,7 @@
         </is>
       </c>
       <c r="E201" s="2" t="n">
-        <v>2641639.21</v>
+        <v>2225236.72</v>
       </c>
     </row>
     <row r="202">
@@ -5490,7 +5490,7 @@
         </is>
       </c>
       <c r="E203" s="2" t="n">
-        <v>39.14</v>
+        <v>38.61</v>
       </c>
     </row>
     <row r="204">
@@ -5515,7 +5515,7 @@
         </is>
       </c>
       <c r="E204" s="2" t="n">
-        <v>43.59</v>
+        <v>38.08</v>
       </c>
     </row>
     <row r="205">
@@ -5540,7 +5540,7 @@
         </is>
       </c>
       <c r="E205" s="2" t="n">
-        <v>1</v>
+        <v>0.8250999999999999</v>
       </c>
     </row>
     <row r="206">
@@ -5640,7 +5640,7 @@
         </is>
       </c>
       <c r="E209" s="2" t="n">
-        <v>2641639.21</v>
+        <v>2225236.72</v>
       </c>
     </row>
     <row r="210">
@@ -5665,7 +5665,7 @@
         </is>
       </c>
       <c r="E210" s="2" t="n">
-        <v>-1446757.06</v>
+        <v>-1401823.44</v>
       </c>
     </row>
     <row r="211">
@@ -5690,7 +5690,7 @@
         </is>
       </c>
       <c r="E211" s="2" t="n">
-        <v>1151598.36</v>
+        <v>847421.75</v>
       </c>
     </row>
     <row r="212">
@@ -5940,7 +5940,7 @@
         </is>
       </c>
       <c r="E221" s="2" t="n">
-        <v>2641639.21</v>
+        <v>2225236.72</v>
       </c>
     </row>
     <row r="222">
@@ -5965,7 +5965,7 @@
         </is>
       </c>
       <c r="E222" s="2" t="n">
-        <v>-1446757.06</v>
+        <v>-1401823.44</v>
       </c>
     </row>
     <row r="223">
@@ -5990,7 +5990,7 @@
         </is>
       </c>
       <c r="E223" s="2" t="n">
-        <v>1151598.36</v>
+        <v>847421.75</v>
       </c>
     </row>
     <row r="224">
@@ -6001,7 +6001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -6026,7 +6026,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -6065,7 +6065,7 @@
         </is>
       </c>
       <c r="E226" s="2" t="n">
-        <v>3042869.33</v>
+        <v>5905118</v>
       </c>
     </row>
     <row r="227">
@@ -6076,7 +6076,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -6090,7 +6090,7 @@
         </is>
       </c>
       <c r="E227" s="2" t="n">
-        <v>2137417.32</v>
+        <v>5008003.65</v>
       </c>
     </row>
     <row r="228">
@@ -6101,7 +6101,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -6140,7 +6140,7 @@
         </is>
       </c>
       <c r="E229" s="2" t="n">
-        <v>37.41</v>
+        <v>35.76</v>
       </c>
     </row>
     <row r="230">
@@ -6151,7 +6151,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -6165,7 +6165,7 @@
         </is>
       </c>
       <c r="E230" s="2" t="n">
-        <v>10.65</v>
+        <v>28.41</v>
       </c>
     </row>
     <row r="231">
@@ -6176,7 +6176,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -6226,7 +6226,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -6251,7 +6251,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -6290,7 +6290,7 @@
         </is>
       </c>
       <c r="E235" s="2" t="n">
-        <v>2137417.32</v>
+        <v>5008003.65</v>
       </c>
     </row>
     <row r="236">
@@ -6301,7 +6301,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -6315,7 +6315,7 @@
         </is>
       </c>
       <c r="E236" s="2" t="n">
-        <v>-1681883.3</v>
+        <v>-2573153.93</v>
       </c>
     </row>
     <row r="237">
@@ -6326,7 +6326,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -6340,7 +6340,7 @@
         </is>
       </c>
       <c r="E237" s="2" t="n">
-        <v>227545.22</v>
+        <v>1423011.21</v>
       </c>
     </row>
     <row r="238">
@@ -6351,7 +6351,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -6376,7 +6376,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -6401,7 +6401,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -6426,7 +6426,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -6451,7 +6451,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -6476,7 +6476,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -6501,7 +6501,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -6526,7 +6526,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -6551,7 +6551,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -6576,7 +6576,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -6590,7 +6590,7 @@
         </is>
       </c>
       <c r="E247" s="2" t="n">
-        <v>2137417.32</v>
+        <v>5008003.65</v>
       </c>
     </row>
     <row r="248">
@@ -6601,7 +6601,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -6615,7 +6615,7 @@
         </is>
       </c>
       <c r="E248" s="2" t="n">
-        <v>-1681883.3</v>
+        <v>-2573153.93</v>
       </c>
     </row>
     <row r="249">
@@ -6626,7 +6626,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -6640,7 +6640,7 @@
         </is>
       </c>
       <c r="E249" s="2" t="n">
-        <v>227545.22</v>
+        <v>1423011.21</v>
       </c>
     </row>
     <row r="250">
@@ -9970,7 +9970,7 @@
         </is>
       </c>
       <c r="E383" s="2" t="n">
-        <v>2454423.55</v>
+        <v>3312183.57</v>
       </c>
     </row>
     <row r="384">
@@ -10045,7 +10045,7 @@
         </is>
       </c>
       <c r="E386" s="2" t="n">
-        <v>34.27</v>
+        <v>38.86</v>
       </c>
     </row>
     <row r="387">
@@ -10070,7 +10070,7 @@
         </is>
       </c>
       <c r="E387" s="2" t="n">
-        <v>0</v>
+        <v>0.9892</v>
       </c>
     </row>
     <row r="388">
@@ -10170,7 +10170,7 @@
         </is>
       </c>
       <c r="E391" s="2" t="n">
-        <v>2180205.61</v>
+        <v>2824477.1</v>
       </c>
     </row>
     <row r="392">
@@ -10195,7 +10195,7 @@
         </is>
       </c>
       <c r="E392" s="2" t="n">
-        <v>-650050.16</v>
+        <v>-926793.5600000001</v>
       </c>
     </row>
     <row r="393">
@@ -10220,7 +10220,7 @@
         </is>
       </c>
       <c r="E393" s="2" t="n">
-        <v>746305.74</v>
+        <v>1113833.83</v>
       </c>
     </row>
     <row r="394">
@@ -10245,7 +10245,7 @@
         </is>
       </c>
       <c r="E394" s="2" t="n">
-        <v>77668.92</v>
+        <v>112668.92</v>
       </c>
     </row>
     <row r="395">
@@ -10270,7 +10270,7 @@
         </is>
       </c>
       <c r="E395" s="2" t="n">
-        <v>-50484.8</v>
+        <v>-73234.8</v>
       </c>
     </row>
     <row r="396">
@@ -10295,7 +10295,7 @@
         </is>
       </c>
       <c r="E396" s="2" t="n">
-        <v>27184.12</v>
+        <v>39434.12</v>
       </c>
     </row>
     <row r="397">
@@ -10395,7 +10395,7 @@
         </is>
       </c>
       <c r="E400" s="2" t="n">
-        <v>30000</v>
+        <v>208488.53</v>
       </c>
     </row>
     <row r="401">
@@ -10420,7 +10420,7 @@
         </is>
       </c>
       <c r="E401" s="2" t="n">
-        <v>-18900</v>
+        <v>-131347.77</v>
       </c>
     </row>
     <row r="402">
@@ -10445,7 +10445,7 @@
         </is>
       </c>
       <c r="E402" s="2" t="n">
-        <v>11100</v>
+        <v>77140.75999999999</v>
       </c>
     </row>
     <row r="403">
@@ -10470,7 +10470,7 @@
         </is>
       </c>
       <c r="E403" s="2" t="n">
-        <v>2454423.55</v>
+        <v>3312183.57</v>
       </c>
     </row>
     <row r="404">
@@ -10495,7 +10495,7 @@
         </is>
       </c>
       <c r="E404" s="2" t="n">
-        <v>-829357.3100000001</v>
+        <v>-1241298.49</v>
       </c>
     </row>
     <row r="405">
@@ -10520,7 +10520,7 @@
         </is>
       </c>
       <c r="E405" s="2" t="n">
-        <v>841216.53</v>
+        <v>1287035.37</v>
       </c>
     </row>
     <row r="406">
@@ -10531,7 +10531,7 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
@@ -10545,7 +10545,7 @@
         </is>
       </c>
       <c r="E406" s="2" t="n">
-        <v>19120.07</v>
+        <v>17429.85</v>
       </c>
     </row>
     <row r="407">
@@ -10556,7 +10556,7 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
@@ -10570,7 +10570,7 @@
         </is>
       </c>
       <c r="E407" s="2" t="n">
-        <v>0.5311</v>
+        <v>0.4842</v>
       </c>
     </row>
     <row r="408">
@@ -10581,7 +10581,7 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
@@ -10595,7 +10595,7 @@
         </is>
       </c>
       <c r="E408" s="2" t="n">
-        <v>5024268.13</v>
+        <v>5024268.01</v>
       </c>
     </row>
     <row r="409">
@@ -10606,7 +10606,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
@@ -10620,7 +10620,7 @@
         </is>
       </c>
       <c r="E409" s="2" t="n">
-        <v>4114791.7</v>
+        <v>4172319.52</v>
       </c>
     </row>
     <row r="410">
@@ -10631,7 +10631,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
@@ -10656,7 +10656,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
@@ -10681,7 +10681,7 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
@@ -10695,7 +10695,7 @@
         </is>
       </c>
       <c r="E412" s="2" t="n">
-        <v>34.61</v>
+        <v>34.59</v>
       </c>
     </row>
     <row r="413">
@@ -10706,7 +10706,7 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -10731,7 +10731,7 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
@@ -10756,7 +10756,7 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
@@ -10781,7 +10781,7 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
@@ -10806,7 +10806,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -10820,7 +10820,7 @@
         </is>
       </c>
       <c r="E417" s="2" t="n">
-        <v>4114791.7</v>
+        <v>4172319.52</v>
       </c>
     </row>
     <row r="418">
@@ -10831,7 +10831,7 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
@@ -10845,7 +10845,7 @@
         </is>
       </c>
       <c r="E418" s="2" t="n">
-        <v>-2590732.31</v>
+        <v>-2629492.31</v>
       </c>
     </row>
     <row r="419">
@@ -10856,7 +10856,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -10870,7 +10870,7 @@
         </is>
       </c>
       <c r="E419" s="2" t="n">
-        <v>1424309.39</v>
+        <v>1443077.21</v>
       </c>
     </row>
     <row r="420">
@@ -10881,7 +10881,7 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
@@ -10906,7 +10906,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -10931,7 +10931,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -10981,7 +10981,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -11006,7 +11006,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
@@ -11031,7 +11031,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
@@ -11081,7 +11081,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
@@ -11106,7 +11106,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
@@ -11120,7 +11120,7 @@
         </is>
       </c>
       <c r="E429" s="2" t="n">
-        <v>4114791.7</v>
+        <v>4172319.52</v>
       </c>
     </row>
     <row r="430">
@@ -11131,7 +11131,7 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
@@ -11145,7 +11145,7 @@
         </is>
       </c>
       <c r="E430" s="2" t="n">
-        <v>-2590732.31</v>
+        <v>-2629492.31</v>
       </c>
     </row>
     <row r="431">
@@ -11156,7 +11156,7 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>AE_GM</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
@@ -11170,7 +11170,7 @@
         </is>
       </c>
       <c r="E431" s="2" t="n">
-        <v>1424309.39</v>
+        <v>1443077.21</v>
       </c>
     </row>
     <row r="432">
@@ -11270,7 +11270,7 @@
         </is>
       </c>
       <c r="E435" s="2" t="n">
-        <v>15955307.69</v>
+        <v>17705307.01</v>
       </c>
     </row>
     <row r="436">
@@ -11320,7 +11320,7 @@
         </is>
       </c>
       <c r="E437" s="2" t="n">
-        <v>0.5349</v>
+        <v>0</v>
       </c>
     </row>
     <row r="438">
@@ -11370,7 +11370,7 @@
         </is>
       </c>
       <c r="E439" s="2" t="n">
-        <v>3574499.98</v>
+        <v>3651164.47</v>
       </c>
     </row>
     <row r="440">
@@ -11395,7 +11395,7 @@
         </is>
       </c>
       <c r="E440" s="2" t="n">
-        <v>0.8173</v>
+        <v>0.8242</v>
       </c>
     </row>
     <row r="441">
@@ -12020,7 +12020,7 @@
         </is>
       </c>
       <c r="E465" s="2" t="n">
-        <v>0</v>
+        <v>942.91</v>
       </c>
     </row>
     <row r="466">
@@ -12045,7 +12045,7 @@
         </is>
       </c>
       <c r="E466" s="2" t="n">
-        <v>0</v>
+        <v>0.052</v>
       </c>
     </row>
     <row r="467">
@@ -12145,7 +12145,7 @@
         </is>
       </c>
       <c r="E470" s="2" t="n">
-        <v>27.1</v>
+        <v>28.18</v>
       </c>
     </row>
     <row r="471">
@@ -12820,7 +12820,7 @@
         </is>
       </c>
       <c r="E497" s="2" t="n">
-        <v>41.89</v>
+        <v>41.74</v>
       </c>
     </row>
     <row r="498">
@@ -12970,7 +12970,7 @@
         </is>
       </c>
       <c r="E503" s="2" t="n">
-        <v>-2145446.18</v>
+        <v>-2133653.73</v>
       </c>
     </row>
     <row r="504">
@@ -12995,7 +12995,7 @@
         </is>
       </c>
       <c r="E504" s="2" t="n">
-        <v>1558450.5</v>
+        <v>1552100.72</v>
       </c>
     </row>
     <row r="505">
@@ -13270,7 +13270,7 @@
         </is>
       </c>
       <c r="E515" s="2" t="n">
-        <v>-2329721.18</v>
+        <v>-2317928.73</v>
       </c>
     </row>
     <row r="516">
@@ -13295,7 +13295,7 @@
         </is>
       </c>
       <c r="E516" s="2" t="n">
-        <v>1666675.5</v>
+        <v>1660325.72</v>
       </c>
     </row>
     <row r="517">
@@ -13495,7 +13495,7 @@
         </is>
       </c>
       <c r="E524" s="2" t="n">
-        <v>4665135.85</v>
+        <v>4635362.91</v>
       </c>
     </row>
     <row r="525">
@@ -13520,7 +13520,7 @@
         </is>
       </c>
       <c r="E525" s="2" t="n">
-        <v>0.8643999999999999</v>
+        <v>0.8621</v>
       </c>
     </row>
     <row r="526">
@@ -13545,7 +13545,7 @@
         </is>
       </c>
       <c r="E526" s="2" t="n">
-        <v>39.75</v>
+        <v>39.89</v>
       </c>
     </row>
     <row r="527">
@@ -13795,7 +13795,7 @@
         </is>
       </c>
       <c r="E536" s="2" t="n">
-        <v>426454.36</v>
+        <v>36986.16</v>
       </c>
     </row>
     <row r="537">
@@ -13820,7 +13820,7 @@
         </is>
       </c>
       <c r="E537" s="2" t="n">
-        <v>-288647.12</v>
+        <v>-35492.79</v>
       </c>
     </row>
     <row r="538">
@@ -13845,7 +13845,7 @@
         </is>
       </c>
       <c r="E538" s="2" t="n">
-        <v>137807.24</v>
+        <v>1493.37</v>
       </c>
     </row>
     <row r="539">
@@ -13945,7 +13945,7 @@
         </is>
       </c>
       <c r="E542" s="2" t="n">
-        <v>13396161.82</v>
+        <v>13006693.62</v>
       </c>
     </row>
     <row r="543">
@@ -13970,7 +13970,7 @@
         </is>
       </c>
       <c r="E543" s="2" t="n">
-        <v>-8071633.06</v>
+        <v>-7818478.73</v>
       </c>
     </row>
     <row r="544">
@@ -13995,7 +13995,7 @@
         </is>
       </c>
       <c r="E544" s="2" t="n">
-        <v>5324528.76</v>
+        <v>5188214.89</v>
       </c>
     </row>
     <row r="545">
@@ -15445,7 +15445,7 @@
         </is>
       </c>
       <c r="E602" s="2" t="n">
-        <v>0</v>
+        <v>405.77</v>
       </c>
     </row>
     <row r="603">
@@ -15470,7 +15470,7 @@
         </is>
       </c>
       <c r="E603" s="2" t="n">
-        <v>0</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="604">
@@ -16270,7 +16270,7 @@
         </is>
       </c>
       <c r="E635" s="2" t="n">
-        <v>5814009.63</v>
+        <v>5897429.1</v>
       </c>
     </row>
     <row r="636">
@@ -16295,7 +16295,7 @@
         </is>
       </c>
       <c r="E636" s="2" t="n">
-        <v>0.7977</v>
+        <v>0.802</v>
       </c>
     </row>
     <row r="637">
@@ -16320,7 +16320,7 @@
         </is>
       </c>
       <c r="E637" s="2" t="n">
-        <v>38.65</v>
+        <v>38.67</v>
       </c>
     </row>
     <row r="638">
@@ -16420,7 +16420,7 @@
         </is>
       </c>
       <c r="E641" s="2" t="n">
-        <v>16026575.21</v>
+        <v>16008432.98</v>
       </c>
     </row>
     <row r="642">
@@ -16445,7 +16445,7 @@
         </is>
       </c>
       <c r="E642" s="2" t="n">
-        <v>-9470632.619999999</v>
+        <v>-9458840.17</v>
       </c>
     </row>
     <row r="643">
@@ -16470,7 +16470,7 @@
         </is>
       </c>
       <c r="E643" s="2" t="n">
-        <v>6555942.59</v>
+        <v>6549592.81</v>
       </c>
     </row>
     <row r="644">
@@ -16570,7 +16570,7 @@
         </is>
       </c>
       <c r="E647" s="2" t="n">
-        <v>387515.97</v>
+        <v>300331.34</v>
       </c>
     </row>
     <row r="648">
@@ -16595,7 +16595,7 @@
         </is>
       </c>
       <c r="E648" s="2" t="n">
-        <v>-251885.38</v>
+        <v>-195215.37</v>
       </c>
     </row>
     <row r="649">
@@ -16620,7 +16620,7 @@
         </is>
       </c>
       <c r="E649" s="2" t="n">
-        <v>135630.59</v>
+        <v>105115.97</v>
       </c>
     </row>
     <row r="650">
@@ -16720,7 +16720,7 @@
         </is>
       </c>
       <c r="E653" s="2" t="n">
-        <v>17240011.13</v>
+        <v>17134684.27</v>
       </c>
     </row>
     <row r="654">
@@ -16745,7 +16745,7 @@
         </is>
       </c>
       <c r="E654" s="2" t="n">
-        <v>-10577404.62</v>
+        <v>-10508942.16</v>
       </c>
     </row>
     <row r="655">
@@ -16770,7 +16770,7 @@
         </is>
       </c>
       <c r="E655" s="2" t="n">
-        <v>6662606.51</v>
+        <v>6625742.109999999</v>
       </c>
     </row>
     <row r="656">

</xml_diff>